<commit_message>
fix: lich su bao cao
</commit_message>
<xml_diff>
--- a/public/templates/baocaocongtruong_daolo.xlsx
+++ b/public/templates/baocaocongtruong_daolo.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Production Management System\public\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\trant\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4EBF961-16F4-432C-AAED-DA362DF5AFAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{459A1CE6-AB8E-4469-87F7-5892DD491578}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{5C745F27-00A4-4073-9875-97C9D69AA075}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{5C745F27-00A4-4073-9875-97C9D69AA075}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="44">
   <si>
     <t>NHẬT KÝ SẢN XUẤT THEO CA</t>
   </si>
@@ -61,9 +61,6 @@
   </si>
   <si>
     <t>Ca làm việc bình thường.</t>
-  </si>
-  <si>
-    <t>CT Đào lò 1</t>
   </si>
   <si>
     <t>Lò DVVT 30707</t>
@@ -121,9 +118,6 @@
     <t>Ca 3</t>
   </si>
   <si>
-    <t>CT Đào lò 2</t>
-  </si>
-  <si>
     <t>Lò nối TG -30</t>
   </si>
   <si>
@@ -138,6 +132,36 @@
   <si>
     <t>Lò VT -357</t>
   </si>
+  <si>
+    <t>Lò XV mức -35</t>
+  </si>
+  <si>
+    <t>Lò XV mức -355</t>
+  </si>
+  <si>
+    <t>Lò TG mức -296</t>
+  </si>
+  <si>
+    <t>Lò TG mức -297</t>
+  </si>
+  <si>
+    <t>Lò VT -358</t>
+  </si>
+  <si>
+    <t>Lò VT -359</t>
+  </si>
+  <si>
+    <t>Lò nối -51</t>
+  </si>
+  <si>
+    <t>Lò nối -52</t>
+  </si>
+  <si>
+    <t>Đào lò 1</t>
+  </si>
+  <si>
+    <t>Đào lò 2</t>
+  </si>
 </sst>
 </file>
 
@@ -147,7 +171,7 @@
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
     <numFmt numFmtId="165" formatCode="#,##0.0"/>
   </numFmts>
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -233,6 +257,12 @@
       <color theme="0"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="12">
@@ -535,7 +565,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -583,9 +613,6 @@
     <xf numFmtId="0" fontId="10" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="165" fontId="6" fillId="9" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -596,49 +623,7 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="3" fontId="6" fillId="9" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="9" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="9" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="9" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="4" fillId="9" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="4" fillId="9" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="4" fillId="9" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -690,6 +675,42 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="11" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="9" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="9" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="9" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="9" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="9" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="9" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1026,74 +1047,74 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C33E5CFA-3E25-4D2F-BDFC-A7AD5103D39A}">
   <dimension ref="A1:Z290"/>
-  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="13" customWidth="1"/>
     <col min="3" max="5" width="9" customWidth="1"/>
-    <col min="6" max="6" width="17.453125" style="7" customWidth="1"/>
-    <col min="7" max="7" width="9.36328125" style="7" customWidth="1"/>
-    <col min="8" max="10" width="6.08984375" style="7" customWidth="1"/>
-    <col min="11" max="11" width="16.1796875" style="7" customWidth="1"/>
-    <col min="12" max="12" width="8.6328125" style="7" customWidth="1"/>
-    <col min="13" max="15" width="6.6328125" style="7" customWidth="1"/>
-    <col min="16" max="16" width="16.1796875" style="7" customWidth="1"/>
-    <col min="17" max="19" width="6.08984375" style="7" customWidth="1"/>
-    <col min="20" max="21" width="9.6328125" style="7" customWidth="1"/>
-    <col min="22" max="22" width="25.26953125" customWidth="1"/>
-    <col min="23" max="25" width="23.453125" customWidth="1"/>
-    <col min="26" max="26" width="19.90625" customWidth="1"/>
+    <col min="6" max="6" width="17.42578125" style="7" customWidth="1"/>
+    <col min="7" max="7" width="9.42578125" style="7" customWidth="1"/>
+    <col min="8" max="10" width="6.140625" style="7" customWidth="1"/>
+    <col min="11" max="11" width="16.140625" style="7" customWidth="1"/>
+    <col min="12" max="12" width="8.5703125" style="7" customWidth="1"/>
+    <col min="13" max="15" width="6.5703125" style="7" customWidth="1"/>
+    <col min="16" max="16" width="16.140625" style="7" customWidth="1"/>
+    <col min="17" max="19" width="6.140625" style="7" customWidth="1"/>
+    <col min="20" max="21" width="9.5703125" style="7" customWidth="1"/>
+    <col min="22" max="22" width="25.28515625" customWidth="1"/>
+    <col min="23" max="25" width="23.42578125" customWidth="1"/>
+    <col min="26" max="26" width="19.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="37" t="s">
+    <row r="1" spans="1:26" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="22" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="38"/>
-      <c r="C1" s="38"/>
-      <c r="D1" s="38"/>
-      <c r="E1" s="39"/>
-      <c r="F1" s="39"/>
-      <c r="G1" s="39"/>
-      <c r="H1" s="39"/>
-      <c r="I1" s="39"/>
-      <c r="J1" s="39"/>
-      <c r="K1" s="39"/>
-      <c r="L1" s="39"/>
-      <c r="M1" s="39"/>
-      <c r="N1" s="39"/>
-      <c r="O1" s="39"/>
-      <c r="P1" s="39"/>
-      <c r="Q1" s="39"/>
-      <c r="R1" s="39"/>
-      <c r="S1" s="39"/>
-      <c r="T1" s="39"/>
-      <c r="U1" s="39"/>
-      <c r="V1" s="39"/>
-      <c r="W1" s="39"/>
-      <c r="X1" s="39"/>
-      <c r="Y1" s="39"/>
-      <c r="Z1" s="40"/>
-    </row>
-    <row r="2" spans="1:26" ht="26.4" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B1" s="23"/>
+      <c r="C1" s="23"/>
+      <c r="D1" s="23"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
+      <c r="G1" s="24"/>
+      <c r="H1" s="24"/>
+      <c r="I1" s="24"/>
+      <c r="J1" s="24"/>
+      <c r="K1" s="24"/>
+      <c r="L1" s="24"/>
+      <c r="M1" s="24"/>
+      <c r="N1" s="24"/>
+      <c r="O1" s="24"/>
+      <c r="P1" s="24"/>
+      <c r="Q1" s="24"/>
+      <c r="R1" s="24"/>
+      <c r="S1" s="24"/>
+      <c r="T1" s="24"/>
+      <c r="U1" s="24"/>
+      <c r="V1" s="24"/>
+      <c r="W1" s="24"/>
+      <c r="X1" s="24"/>
+      <c r="Y1" s="24"/>
+      <c r="Z1" s="25"/>
+    </row>
+    <row r="2" spans="1:26" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
-      <c r="F2" s="41" t="s">
+      <c r="F2" s="26" t="s">
+        <v>21</v>
+      </c>
+      <c r="G2" s="27"/>
+      <c r="H2" s="27"/>
+      <c r="I2" s="27"/>
+      <c r="J2" s="28"/>
+      <c r="K2" s="26" t="s">
         <v>22</v>
       </c>
-      <c r="G2" s="42"/>
-      <c r="H2" s="42"/>
-      <c r="I2" s="42"/>
-      <c r="J2" s="43"/>
-      <c r="K2" s="41" t="s">
-        <v>23</v>
-      </c>
-      <c r="L2" s="42"/>
-      <c r="M2" s="42"/>
-      <c r="N2" s="42"/>
-      <c r="O2" s="43"/>
+      <c r="L2" s="27"/>
+      <c r="M2" s="27"/>
+      <c r="N2" s="27"/>
+      <c r="O2" s="28"/>
       <c r="P2" s="8"/>
       <c r="Q2" s="8"/>
       <c r="R2" s="8"/>
@@ -1106,371 +1127,502 @@
       <c r="Y2" s="1"/>
       <c r="Z2" s="1"/>
     </row>
-    <row r="3" spans="1:26" ht="39" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:26" ht="39" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="31" t="s">
+      <c r="C3" s="43" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" s="44"/>
+      <c r="E3" s="45"/>
+      <c r="F3" s="10" t="s">
         <v>13</v>
-      </c>
-      <c r="D3" s="32"/>
-      <c r="E3" s="33"/>
-      <c r="F3" s="10" t="s">
-        <v>14</v>
       </c>
       <c r="G3" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="H3" s="44" t="s">
-        <v>18</v>
-      </c>
-      <c r="I3" s="44"/>
-      <c r="J3" s="44"/>
+      <c r="H3" s="29" t="s">
+        <v>17</v>
+      </c>
+      <c r="I3" s="29"/>
+      <c r="J3" s="29"/>
       <c r="K3" s="13" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="L3" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="M3" s="45" t="s">
-        <v>17</v>
-      </c>
-      <c r="N3" s="45"/>
-      <c r="O3" s="45"/>
+      <c r="M3" s="30" t="s">
+        <v>16</v>
+      </c>
+      <c r="N3" s="30"/>
+      <c r="O3" s="30"/>
       <c r="P3" s="12" t="s">
-        <v>21</v>
-      </c>
-      <c r="Q3" s="46" t="s">
-        <v>26</v>
-      </c>
-      <c r="R3" s="47"/>
-      <c r="S3" s="48"/>
-      <c r="T3" s="49" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q3" s="31" t="s">
+        <v>25</v>
+      </c>
+      <c r="R3" s="32"/>
+      <c r="S3" s="33"/>
+      <c r="T3" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="U3" s="50"/>
-      <c r="V3" s="51"/>
-      <c r="W3" s="52" t="s">
+      <c r="U3" s="35"/>
+      <c r="V3" s="36"/>
+      <c r="W3" s="37" t="s">
         <v>6</v>
       </c>
-      <c r="X3" s="53"/>
-      <c r="Y3" s="54"/>
+      <c r="X3" s="38"/>
+      <c r="Y3" s="39"/>
       <c r="Z3" s="9" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:26" s="14" customFormat="1" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:26" s="14" customFormat="1" ht="20.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C4" s="15" t="s">
+        <v>26</v>
+      </c>
+      <c r="D4" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="D4" s="15" t="s">
+      <c r="E4" s="15" t="s">
         <v>28</v>
-      </c>
-      <c r="E4" s="15" t="s">
-        <v>29</v>
       </c>
       <c r="F4" s="15"/>
       <c r="G4" s="15"/>
       <c r="H4" s="15" t="s">
+        <v>26</v>
+      </c>
+      <c r="I4" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="I4" s="15" t="s">
+      <c r="J4" s="15" t="s">
         <v>28</v>
-      </c>
-      <c r="J4" s="15" t="s">
-        <v>29</v>
       </c>
       <c r="K4" s="15"/>
       <c r="L4" s="15"/>
       <c r="M4" s="15" t="s">
+        <v>26</v>
+      </c>
+      <c r="N4" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="N4" s="15" t="s">
+      <c r="O4" s="15" t="s">
         <v>28</v>
-      </c>
-      <c r="O4" s="15" t="s">
-        <v>29</v>
       </c>
       <c r="P4" s="16"/>
       <c r="Q4" s="15" t="s">
+        <v>26</v>
+      </c>
+      <c r="R4" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="R4" s="15" t="s">
+      <c r="S4" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="S4" s="15" t="s">
+      <c r="T4" s="15" t="s">
+        <v>26</v>
+      </c>
+      <c r="U4" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="V4" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="W4" s="15" t="s">
+        <v>26</v>
+      </c>
+      <c r="X4" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y4" s="15" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="5" spans="1:26" s="20" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A5" s="49">
+        <v>46204</v>
+      </c>
+      <c r="B5" s="40" t="s">
+        <v>42</v>
+      </c>
+      <c r="C5" s="40">
+        <v>70</v>
+      </c>
+      <c r="D5" s="40">
+        <v>70</v>
+      </c>
+      <c r="E5" s="46">
+        <v>71</v>
+      </c>
+      <c r="F5" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="G5" s="17">
+        <v>12.1</v>
+      </c>
+      <c r="H5" s="17">
+        <v>2</v>
+      </c>
+      <c r="I5" s="17">
+        <v>4</v>
+      </c>
+      <c r="J5" s="17">
+        <v>3</v>
+      </c>
+      <c r="K5" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="L5" s="17">
+        <v>16</v>
+      </c>
+      <c r="M5" s="17">
+        <v>3</v>
+      </c>
+      <c r="N5" s="17">
+        <v>2</v>
+      </c>
+      <c r="O5" s="17">
+        <v>2</v>
+      </c>
+      <c r="P5" s="17" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q5" s="17">
+        <v>2</v>
+      </c>
+      <c r="R5" s="17">
+        <v>3</v>
+      </c>
+      <c r="S5" s="17">
+        <v>2</v>
+      </c>
+      <c r="T5" s="17"/>
+      <c r="U5" s="17"/>
+      <c r="V5" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="W5" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="X5" s="19" t="s">
+        <v>9</v>
+      </c>
+      <c r="Y5" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="Z5" s="19"/>
+    </row>
+    <row r="6" spans="1:26" s="20" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A6" s="50"/>
+      <c r="B6" s="41"/>
+      <c r="C6" s="41"/>
+      <c r="D6" s="41"/>
+      <c r="E6" s="47"/>
+      <c r="F6" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="G6" s="17">
+        <v>11.9</v>
+      </c>
+      <c r="H6" s="17">
+        <v>3</v>
+      </c>
+      <c r="I6" s="17">
+        <v>3</v>
+      </c>
+      <c r="J6" s="17">
+        <v>3</v>
+      </c>
+      <c r="K6" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="L6" s="17">
+        <v>14</v>
+      </c>
+      <c r="M6" s="17">
+        <v>3</v>
+      </c>
+      <c r="N6" s="17">
+        <v>2</v>
+      </c>
+      <c r="O6" s="17">
+        <v>2</v>
+      </c>
+      <c r="P6" s="17" t="s">
+        <v>36</v>
+      </c>
+      <c r="Q6" s="17">
+        <v>2</v>
+      </c>
+      <c r="R6" s="17">
+        <v>3</v>
+      </c>
+      <c r="S6" s="17">
+        <v>2</v>
+      </c>
+      <c r="T6" s="17"/>
+      <c r="U6" s="17"/>
+      <c r="V6" s="21"/>
+      <c r="W6" s="21"/>
+      <c r="X6" s="21"/>
+      <c r="Y6" s="19" t="s">
+        <v>9</v>
+      </c>
+      <c r="Z6" s="19"/>
+    </row>
+    <row r="7" spans="1:26" s="20" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="50"/>
+      <c r="B7" s="42"/>
+      <c r="C7" s="42"/>
+      <c r="D7" s="42"/>
+      <c r="E7" s="48"/>
+      <c r="F7" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="G7" s="17">
+        <v>8.1</v>
+      </c>
+      <c r="H7" s="17">
+        <v>4</v>
+      </c>
+      <c r="I7" s="17">
+        <v>2</v>
+      </c>
+      <c r="J7" s="17">
+        <v>3</v>
+      </c>
+      <c r="K7" s="17" t="s">
+        <v>35</v>
+      </c>
+      <c r="L7" s="17">
+        <v>14</v>
+      </c>
+      <c r="M7" s="17">
+        <v>3</v>
+      </c>
+      <c r="N7" s="17">
+        <v>2</v>
+      </c>
+      <c r="O7" s="17">
+        <v>2</v>
+      </c>
+      <c r="P7" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q7" s="17">
+        <v>2</v>
+      </c>
+      <c r="R7" s="17">
+        <v>3</v>
+      </c>
+      <c r="S7" s="17">
+        <v>2</v>
+      </c>
+      <c r="T7" s="17"/>
+      <c r="U7" s="17"/>
+      <c r="V7" s="21"/>
+      <c r="W7" s="21"/>
+      <c r="X7" s="21"/>
+      <c r="Y7" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="Z7" s="19"/>
+    </row>
+    <row r="8" spans="1:26" s="20" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A8" s="50"/>
+      <c r="B8" s="40" t="s">
+        <v>43</v>
+      </c>
+      <c r="C8" s="40">
+        <v>71</v>
+      </c>
+      <c r="D8" s="40">
+        <v>71</v>
+      </c>
+      <c r="E8" s="46">
+        <v>71</v>
+      </c>
+      <c r="F8" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="T4" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="U4" s="15" t="s">
-        <v>28</v>
-      </c>
-      <c r="V4" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="W4" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="X4" s="15" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y4" s="15" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="5" spans="1:26" s="21" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="28">
-        <v>46204</v>
-      </c>
-      <c r="B5" s="25" t="s">
-        <v>11</v>
-      </c>
-      <c r="C5" s="17"/>
-      <c r="D5" s="17"/>
-      <c r="E5" s="34">
-        <v>71</v>
-      </c>
-      <c r="F5" s="14" t="s">
-        <v>12</v>
-      </c>
-      <c r="G5" s="18">
-        <v>12.1</v>
-      </c>
-      <c r="H5" s="18"/>
-      <c r="I5" s="18"/>
-      <c r="J5" s="18"/>
-      <c r="K5" s="18" t="s">
-        <v>19</v>
-      </c>
-      <c r="L5" s="18">
+      <c r="G8" s="17">
+        <v>10</v>
+      </c>
+      <c r="H8" s="17">
+        <v>2</v>
+      </c>
+      <c r="I8" s="17">
+        <v>4</v>
+      </c>
+      <c r="J8" s="17">
+        <v>3</v>
+      </c>
+      <c r="K8" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="L8" s="17">
         <v>16</v>
       </c>
-      <c r="M5" s="18"/>
-      <c r="N5" s="18"/>
-      <c r="O5" s="18">
+      <c r="M8" s="17">
+        <v>3</v>
+      </c>
+      <c r="N8" s="17">
         <v>2</v>
       </c>
-      <c r="P5" s="18" t="s">
+      <c r="O8" s="17">
+        <v>2</v>
+      </c>
+      <c r="P8" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q8" s="17">
+        <v>2</v>
+      </c>
+      <c r="R8" s="17">
+        <v>2</v>
+      </c>
+      <c r="S8" s="17">
+        <v>2</v>
+      </c>
+      <c r="T8" s="17"/>
+      <c r="U8" s="17"/>
+      <c r="V8" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="Q5" s="18"/>
-      <c r="R5" s="18"/>
-      <c r="S5" s="18">
+      <c r="W8" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="X8" s="19" t="s">
+        <v>9</v>
+      </c>
+      <c r="Y8" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="Z8" s="19"/>
+    </row>
+    <row r="9" spans="1:26" s="20" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A9" s="50"/>
+      <c r="B9" s="41"/>
+      <c r="C9" s="41"/>
+      <c r="D9" s="41"/>
+      <c r="E9" s="47"/>
+      <c r="F9" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="G9" s="17">
+        <v>8</v>
+      </c>
+      <c r="H9" s="17">
+        <v>3</v>
+      </c>
+      <c r="I9" s="17">
+        <v>4</v>
+      </c>
+      <c r="J9" s="17">
+        <v>3</v>
+      </c>
+      <c r="K9" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="L9" s="17">
+        <v>17</v>
+      </c>
+      <c r="M9" s="17">
+        <v>3</v>
+      </c>
+      <c r="N9" s="17">
         <v>2</v>
       </c>
-      <c r="T5" s="18"/>
-      <c r="U5" s="18"/>
-      <c r="V5" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="W5" s="20" t="s">
+      <c r="O9" s="17">
+        <v>2</v>
+      </c>
+      <c r="P9" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q9" s="17">
+        <v>22</v>
+      </c>
+      <c r="R9" s="17">
+        <v>2</v>
+      </c>
+      <c r="S9" s="17">
+        <v>2</v>
+      </c>
+      <c r="T9" s="17"/>
+      <c r="U9" s="17"/>
+      <c r="V9" s="21"/>
+      <c r="W9" s="21"/>
+      <c r="X9" s="21"/>
+      <c r="Y9" s="19" t="s">
+        <v>9</v>
+      </c>
+      <c r="Z9" s="19"/>
+    </row>
+    <row r="10" spans="1:26" s="20" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="51"/>
+      <c r="B10" s="42"/>
+      <c r="C10" s="42"/>
+      <c r="D10" s="42"/>
+      <c r="E10" s="48"/>
+      <c r="F10" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="G10" s="17">
+        <v>7</v>
+      </c>
+      <c r="H10" s="17">
+        <v>4</v>
+      </c>
+      <c r="I10" s="17">
+        <v>3</v>
+      </c>
+      <c r="J10" s="17">
+        <v>3</v>
+      </c>
+      <c r="K10" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="L10" s="17">
+        <v>17</v>
+      </c>
+      <c r="M10" s="17">
+        <v>2</v>
+      </c>
+      <c r="N10" s="17">
+        <v>2</v>
+      </c>
+      <c r="O10" s="17">
+        <v>2</v>
+      </c>
+      <c r="P10" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q10" s="17">
+        <v>2</v>
+      </c>
+      <c r="R10" s="17">
+        <v>2</v>
+      </c>
+      <c r="S10" s="17">
+        <v>2</v>
+      </c>
+      <c r="T10" s="17"/>
+      <c r="U10" s="17"/>
+      <c r="V10" s="21"/>
+      <c r="W10" s="21"/>
+      <c r="X10" s="21"/>
+      <c r="Y10" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="X5" s="20" t="s">
-        <v>9</v>
-      </c>
-      <c r="Y5" s="20" t="s">
-        <v>8</v>
-      </c>
-      <c r="Z5" s="20"/>
-    </row>
-    <row r="6" spans="1:26" s="21" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="29"/>
-      <c r="B6" s="26"/>
-      <c r="C6" s="22"/>
-      <c r="D6" s="22"/>
-      <c r="E6" s="35"/>
-      <c r="F6" s="14" t="s">
-        <v>15</v>
-      </c>
-      <c r="G6" s="18">
-        <v>11.9</v>
-      </c>
-      <c r="H6" s="18"/>
-      <c r="I6" s="18"/>
-      <c r="J6" s="18"/>
-      <c r="K6" s="18"/>
-      <c r="L6" s="18"/>
-      <c r="M6" s="18"/>
-      <c r="N6" s="18"/>
-      <c r="O6" s="18"/>
-      <c r="P6" s="18"/>
-      <c r="Q6" s="18"/>
-      <c r="R6" s="18"/>
-      <c r="S6" s="18"/>
-      <c r="T6" s="18"/>
-      <c r="U6" s="18"/>
-      <c r="V6" s="23"/>
-      <c r="W6" s="23"/>
-      <c r="X6" s="23"/>
-      <c r="Y6" s="20" t="s">
-        <v>9</v>
-      </c>
-      <c r="Z6" s="20"/>
-    </row>
-    <row r="7" spans="1:26" s="21" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="30"/>
-      <c r="B7" s="27"/>
-      <c r="C7" s="24"/>
-      <c r="D7" s="24"/>
-      <c r="E7" s="36"/>
-      <c r="F7" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="G7" s="18">
-        <v>8.1</v>
-      </c>
-      <c r="H7" s="18"/>
-      <c r="I7" s="18"/>
-      <c r="J7" s="18"/>
-      <c r="K7" s="18"/>
-      <c r="L7" s="18"/>
-      <c r="M7" s="18"/>
-      <c r="N7" s="18"/>
-      <c r="O7" s="18"/>
-      <c r="P7" s="18"/>
-      <c r="Q7" s="18"/>
-      <c r="R7" s="18"/>
-      <c r="S7" s="18"/>
-      <c r="T7" s="18"/>
-      <c r="U7" s="18"/>
-      <c r="V7" s="23"/>
-      <c r="W7" s="23"/>
-      <c r="X7" s="23"/>
-      <c r="Y7" s="20" t="s">
-        <v>10</v>
-      </c>
-      <c r="Z7" s="20"/>
-    </row>
-    <row r="8" spans="1:26" s="21" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="28">
-        <v>46204</v>
-      </c>
-      <c r="B8" s="25" t="s">
-        <v>30</v>
-      </c>
-      <c r="C8" s="17"/>
-      <c r="D8" s="17"/>
-      <c r="E8" s="34">
-        <v>71</v>
-      </c>
-      <c r="F8" s="14" t="s">
-        <v>31</v>
-      </c>
-      <c r="G8" s="18">
-        <v>10</v>
-      </c>
-      <c r="H8" s="18"/>
-      <c r="I8" s="18"/>
-      <c r="J8" s="18"/>
-      <c r="K8" s="18" t="s">
-        <v>34</v>
-      </c>
-      <c r="L8" s="18">
-        <v>16</v>
-      </c>
-      <c r="M8" s="18"/>
-      <c r="N8" s="18"/>
-      <c r="O8" s="18">
-        <v>2</v>
-      </c>
-      <c r="P8" s="18" t="s">
-        <v>35</v>
-      </c>
-      <c r="Q8" s="18"/>
-      <c r="R8" s="18"/>
-      <c r="S8" s="18">
-        <v>2</v>
-      </c>
-      <c r="T8" s="18"/>
-      <c r="U8" s="18"/>
-      <c r="V8" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="W8" s="20" t="s">
-        <v>10</v>
-      </c>
-      <c r="X8" s="20" t="s">
-        <v>9</v>
-      </c>
-      <c r="Y8" s="20" t="s">
-        <v>8</v>
-      </c>
-      <c r="Z8" s="20"/>
-    </row>
-    <row r="9" spans="1:26" s="21" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="29"/>
-      <c r="B9" s="26"/>
-      <c r="C9" s="22"/>
-      <c r="D9" s="22"/>
-      <c r="E9" s="35"/>
-      <c r="F9" s="14" t="s">
-        <v>32</v>
-      </c>
-      <c r="G9" s="18">
-        <v>8</v>
-      </c>
-      <c r="H9" s="18"/>
-      <c r="I9" s="18"/>
-      <c r="J9" s="18"/>
-      <c r="K9" s="18"/>
-      <c r="L9" s="18"/>
-      <c r="M9" s="18"/>
-      <c r="N9" s="18"/>
-      <c r="O9" s="18"/>
-      <c r="P9" s="18"/>
-      <c r="Q9" s="18"/>
-      <c r="R9" s="18"/>
-      <c r="S9" s="18"/>
-      <c r="T9" s="18"/>
-      <c r="U9" s="18"/>
-      <c r="V9" s="23"/>
-      <c r="W9" s="23"/>
-      <c r="X9" s="23"/>
-      <c r="Y9" s="20" t="s">
-        <v>9</v>
-      </c>
-      <c r="Z9" s="20"/>
-    </row>
-    <row r="10" spans="1:26" s="21" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="30"/>
-      <c r="B10" s="27"/>
-      <c r="C10" s="24"/>
-      <c r="D10" s="24"/>
-      <c r="E10" s="36"/>
-      <c r="F10" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="G10" s="18">
-        <v>7</v>
-      </c>
-      <c r="H10" s="18"/>
-      <c r="I10" s="18"/>
-      <c r="J10" s="18"/>
-      <c r="K10" s="18"/>
-      <c r="L10" s="18"/>
-      <c r="M10" s="18"/>
-      <c r="N10" s="18"/>
-      <c r="O10" s="18"/>
-      <c r="P10" s="18"/>
-      <c r="Q10" s="18"/>
-      <c r="R10" s="18"/>
-      <c r="S10" s="18"/>
-      <c r="T10" s="18"/>
-      <c r="U10" s="18"/>
-      <c r="V10" s="23"/>
-      <c r="W10" s="23"/>
-      <c r="X10" s="23"/>
-      <c r="Y10" s="20" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="11" spans="1:26" x14ac:dyDescent="0.35">
+      <c r="Z10" s="19"/>
+    </row>
+    <row r="11" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A11" s="6"/>
       <c r="B11" s="6"/>
       <c r="C11" s="6"/>
@@ -1498,7 +1650,7 @@
       <c r="Y11" s="4"/>
       <c r="Z11" s="5"/>
     </row>
-    <row r="12" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A12" s="6"/>
       <c r="B12" s="6"/>
       <c r="C12" s="6"/>
@@ -1526,7 +1678,7 @@
       <c r="Y12" s="4"/>
       <c r="Z12" s="5"/>
     </row>
-    <row r="13" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A13" s="6"/>
       <c r="B13" s="6"/>
       <c r="C13" s="6"/>
@@ -1554,7 +1706,7 @@
       <c r="Y13" s="4"/>
       <c r="Z13" s="5"/>
     </row>
-    <row r="14" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A14" s="6"/>
       <c r="B14" s="6"/>
       <c r="C14" s="6"/>
@@ -1582,7 +1734,7 @@
       <c r="Y14" s="4"/>
       <c r="Z14" s="5"/>
     </row>
-    <row r="15" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A15" s="6"/>
       <c r="B15" s="6"/>
       <c r="C15" s="6"/>
@@ -1610,7 +1762,7 @@
       <c r="Y15" s="4"/>
       <c r="Z15" s="5"/>
     </row>
-    <row r="16" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A16" s="6"/>
       <c r="B16" s="6"/>
       <c r="C16" s="6"/>
@@ -1638,7 +1790,7 @@
       <c r="Y16" s="4"/>
       <c r="Z16" s="5"/>
     </row>
-    <row r="17" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A17" s="6"/>
       <c r="B17" s="6"/>
       <c r="C17" s="6"/>
@@ -1666,7 +1818,7 @@
       <c r="Y17" s="4"/>
       <c r="Z17" s="5"/>
     </row>
-    <row r="18" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A18" s="6"/>
       <c r="B18" s="6"/>
       <c r="C18" s="6"/>
@@ -1694,7 +1846,7 @@
       <c r="Y18" s="4"/>
       <c r="Z18" s="5"/>
     </row>
-    <row r="19" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A19" s="6"/>
       <c r="B19" s="6"/>
       <c r="C19" s="6"/>
@@ -1722,7 +1874,7 @@
       <c r="Y19" s="4"/>
       <c r="Z19" s="5"/>
     </row>
-    <row r="20" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A20" s="6"/>
       <c r="B20" s="6"/>
       <c r="C20" s="6"/>
@@ -1750,7 +1902,7 @@
       <c r="Y20" s="4"/>
       <c r="Z20" s="5"/>
     </row>
-    <row r="21" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A21" s="6"/>
       <c r="B21" s="6"/>
       <c r="C21" s="6"/>
@@ -1778,7 +1930,7 @@
       <c r="Y21" s="4"/>
       <c r="Z21" s="5"/>
     </row>
-    <row r="22" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A22" s="6"/>
       <c r="B22" s="6"/>
       <c r="C22" s="6"/>
@@ -1806,7 +1958,7 @@
       <c r="Y22" s="4"/>
       <c r="Z22" s="5"/>
     </row>
-    <row r="23" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A23" s="6"/>
       <c r="B23" s="6"/>
       <c r="C23" s="6"/>
@@ -1834,7 +1986,7 @@
       <c r="Y23" s="4"/>
       <c r="Z23" s="5"/>
     </row>
-    <row r="24" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A24" s="6"/>
       <c r="B24" s="6"/>
       <c r="C24" s="6"/>
@@ -1862,7 +2014,7 @@
       <c r="Y24" s="4"/>
       <c r="Z24" s="5"/>
     </row>
-    <row r="25" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A25" s="6"/>
       <c r="B25" s="6"/>
       <c r="C25" s="6"/>
@@ -1890,7 +2042,7 @@
       <c r="Y25" s="4"/>
       <c r="Z25" s="5"/>
     </row>
-    <row r="26" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A26" s="6"/>
       <c r="B26" s="6"/>
       <c r="C26" s="6"/>
@@ -1918,7 +2070,7 @@
       <c r="Y26" s="4"/>
       <c r="Z26" s="5"/>
     </row>
-    <row r="27" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A27" s="6"/>
       <c r="B27" s="6"/>
       <c r="C27" s="6"/>
@@ -1946,7 +2098,7 @@
       <c r="Y27" s="4"/>
       <c r="Z27" s="5"/>
     </row>
-    <row r="28" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A28" s="6"/>
       <c r="B28" s="6"/>
       <c r="C28" s="6"/>
@@ -1974,7 +2126,7 @@
       <c r="Y28" s="4"/>
       <c r="Z28" s="5"/>
     </row>
-    <row r="29" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A29" s="6"/>
       <c r="B29" s="6"/>
       <c r="C29" s="6"/>
@@ -2002,7 +2154,7 @@
       <c r="Y29" s="4"/>
       <c r="Z29" s="5"/>
     </row>
-    <row r="30" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A30" s="6"/>
       <c r="B30" s="6"/>
       <c r="C30" s="6"/>
@@ -2030,7 +2182,7 @@
       <c r="Y30" s="4"/>
       <c r="Z30" s="5"/>
     </row>
-    <row r="31" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A31" s="6"/>
       <c r="B31" s="6"/>
       <c r="C31" s="6"/>
@@ -2058,7 +2210,7 @@
       <c r="Y31" s="4"/>
       <c r="Z31" s="5"/>
     </row>
-    <row r="32" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A32" s="6"/>
       <c r="B32" s="6"/>
       <c r="C32" s="6"/>
@@ -2086,7 +2238,7 @@
       <c r="Y32" s="4"/>
       <c r="Z32" s="5"/>
     </row>
-    <row r="33" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A33" s="6"/>
       <c r="B33" s="6"/>
       <c r="C33" s="6"/>
@@ -2114,7 +2266,7 @@
       <c r="Y33" s="4"/>
       <c r="Z33" s="5"/>
     </row>
-    <row r="34" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A34" s="6"/>
       <c r="B34" s="6"/>
       <c r="C34" s="6"/>
@@ -2142,7 +2294,7 @@
       <c r="Y34" s="4"/>
       <c r="Z34" s="5"/>
     </row>
-    <row r="35" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A35" s="6"/>
       <c r="B35" s="6"/>
       <c r="C35" s="6"/>
@@ -2170,7 +2322,7 @@
       <c r="Y35" s="4"/>
       <c r="Z35" s="5"/>
     </row>
-    <row r="36" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A36" s="6"/>
       <c r="B36" s="6"/>
       <c r="C36" s="6"/>
@@ -2198,7 +2350,7 @@
       <c r="Y36" s="4"/>
       <c r="Z36" s="5"/>
     </row>
-    <row r="37" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A37" s="6"/>
       <c r="B37" s="6"/>
       <c r="C37" s="6"/>
@@ -2226,7 +2378,7 @@
       <c r="Y37" s="4"/>
       <c r="Z37" s="5"/>
     </row>
-    <row r="38" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A38" s="6"/>
       <c r="B38" s="6"/>
       <c r="C38" s="6"/>
@@ -2254,7 +2406,7 @@
       <c r="Y38" s="4"/>
       <c r="Z38" s="5"/>
     </row>
-    <row r="39" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A39" s="6"/>
       <c r="B39" s="6"/>
       <c r="C39" s="6"/>
@@ -2282,7 +2434,7 @@
       <c r="Y39" s="4"/>
       <c r="Z39" s="5"/>
     </row>
-    <row r="40" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A40" s="6"/>
       <c r="B40" s="6"/>
       <c r="C40" s="6"/>
@@ -2310,7 +2462,7 @@
       <c r="Y40" s="4"/>
       <c r="Z40" s="5"/>
     </row>
-    <row r="41" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A41" s="6"/>
       <c r="B41" s="6"/>
       <c r="C41" s="6"/>
@@ -2338,7 +2490,7 @@
       <c r="Y41" s="4"/>
       <c r="Z41" s="5"/>
     </row>
-    <row r="42" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A42" s="6"/>
       <c r="B42" s="6"/>
       <c r="C42" s="6"/>
@@ -2366,7 +2518,7 @@
       <c r="Y42" s="4"/>
       <c r="Z42" s="5"/>
     </row>
-    <row r="43" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A43" s="6"/>
       <c r="B43" s="6"/>
       <c r="C43" s="6"/>
@@ -2394,7 +2546,7 @@
       <c r="Y43" s="4"/>
       <c r="Z43" s="5"/>
     </row>
-    <row r="44" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A44" s="6"/>
       <c r="B44" s="6"/>
       <c r="C44" s="6"/>
@@ -2422,7 +2574,7 @@
       <c r="Y44" s="4"/>
       <c r="Z44" s="5"/>
     </row>
-    <row r="45" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A45" s="6"/>
       <c r="B45" s="6"/>
       <c r="C45" s="6"/>
@@ -2450,7 +2602,7 @@
       <c r="Y45" s="4"/>
       <c r="Z45" s="5"/>
     </row>
-    <row r="46" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A46" s="6"/>
       <c r="B46" s="6"/>
       <c r="C46" s="6"/>
@@ -2478,7 +2630,7 @@
       <c r="Y46" s="4"/>
       <c r="Z46" s="5"/>
     </row>
-    <row r="47" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A47" s="6"/>
       <c r="B47" s="6"/>
       <c r="C47" s="6"/>
@@ -2506,7 +2658,7 @@
       <c r="Y47" s="4"/>
       <c r="Z47" s="5"/>
     </row>
-    <row r="48" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A48" s="6"/>
       <c r="B48" s="6"/>
       <c r="C48" s="6"/>
@@ -2534,7 +2686,7 @@
       <c r="Y48" s="4"/>
       <c r="Z48" s="5"/>
     </row>
-    <row r="49" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A49" s="6"/>
       <c r="B49" s="6"/>
       <c r="C49" s="6"/>
@@ -2562,7 +2714,7 @@
       <c r="Y49" s="4"/>
       <c r="Z49" s="5"/>
     </row>
-    <row r="50" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A50" s="6"/>
       <c r="B50" s="6"/>
       <c r="C50" s="6"/>
@@ -2590,7 +2742,7 @@
       <c r="Y50" s="4"/>
       <c r="Z50" s="5"/>
     </row>
-    <row r="51" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A51" s="6"/>
       <c r="B51" s="6"/>
       <c r="C51" s="6"/>
@@ -2618,7 +2770,7 @@
       <c r="Y51" s="4"/>
       <c r="Z51" s="5"/>
     </row>
-    <row r="52" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A52" s="6"/>
       <c r="B52" s="6"/>
       <c r="C52" s="6"/>
@@ -2646,7 +2798,7 @@
       <c r="Y52" s="4"/>
       <c r="Z52" s="5"/>
     </row>
-    <row r="53" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A53" s="6"/>
       <c r="B53" s="6"/>
       <c r="C53" s="6"/>
@@ -2674,7 +2826,7 @@
       <c r="Y53" s="4"/>
       <c r="Z53" s="5"/>
     </row>
-    <row r="54" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A54" s="6"/>
       <c r="B54" s="6"/>
       <c r="C54" s="6"/>
@@ -2702,7 +2854,7 @@
       <c r="Y54" s="4"/>
       <c r="Z54" s="5"/>
     </row>
-    <row r="55" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A55" s="6"/>
       <c r="B55" s="6"/>
       <c r="C55" s="6"/>
@@ -2730,7 +2882,7 @@
       <c r="Y55" s="4"/>
       <c r="Z55" s="5"/>
     </row>
-    <row r="56" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A56" s="6"/>
       <c r="B56" s="6"/>
       <c r="C56" s="6"/>
@@ -2758,7 +2910,7 @@
       <c r="Y56" s="4"/>
       <c r="Z56" s="5"/>
     </row>
-    <row r="57" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A57" s="6"/>
       <c r="B57" s="6"/>
       <c r="C57" s="6"/>
@@ -2786,7 +2938,7 @@
       <c r="Y57" s="4"/>
       <c r="Z57" s="5"/>
     </row>
-    <row r="58" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A58" s="6"/>
       <c r="B58" s="6"/>
       <c r="C58" s="6"/>
@@ -2814,7 +2966,7 @@
       <c r="Y58" s="4"/>
       <c r="Z58" s="5"/>
     </row>
-    <row r="59" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A59" s="6"/>
       <c r="B59" s="6"/>
       <c r="C59" s="6"/>
@@ -2842,7 +2994,7 @@
       <c r="Y59" s="4"/>
       <c r="Z59" s="5"/>
     </row>
-    <row r="60" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A60" s="6"/>
       <c r="B60" s="6"/>
       <c r="C60" s="6"/>
@@ -2870,7 +3022,7 @@
       <c r="Y60" s="4"/>
       <c r="Z60" s="5"/>
     </row>
-    <row r="61" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A61" s="6"/>
       <c r="B61" s="6"/>
       <c r="C61" s="6"/>
@@ -2898,7 +3050,7 @@
       <c r="Y61" s="4"/>
       <c r="Z61" s="5"/>
     </row>
-    <row r="62" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A62" s="6"/>
       <c r="B62" s="6"/>
       <c r="C62" s="6"/>
@@ -2926,7 +3078,7 @@
       <c r="Y62" s="4"/>
       <c r="Z62" s="5"/>
     </row>
-    <row r="63" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A63" s="6"/>
       <c r="B63" s="6"/>
       <c r="C63" s="6"/>
@@ -2954,7 +3106,7 @@
       <c r="Y63" s="4"/>
       <c r="Z63" s="5"/>
     </row>
-    <row r="64" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A64" s="6"/>
       <c r="B64" s="6"/>
       <c r="C64" s="6"/>
@@ -2982,7 +3134,7 @@
       <c r="Y64" s="4"/>
       <c r="Z64" s="5"/>
     </row>
-    <row r="65" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A65" s="6"/>
       <c r="B65" s="6"/>
       <c r="C65" s="6"/>
@@ -3010,7 +3162,7 @@
       <c r="Y65" s="4"/>
       <c r="Z65" s="5"/>
     </row>
-    <row r="66" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A66" s="6"/>
       <c r="B66" s="6"/>
       <c r="C66" s="6"/>
@@ -3038,7 +3190,7 @@
       <c r="Y66" s="4"/>
       <c r="Z66" s="5"/>
     </row>
-    <row r="67" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A67" s="6"/>
       <c r="B67" s="6"/>
       <c r="C67" s="6"/>
@@ -3066,7 +3218,7 @@
       <c r="Y67" s="4"/>
       <c r="Z67" s="5"/>
     </row>
-    <row r="68" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A68" s="6"/>
       <c r="B68" s="6"/>
       <c r="C68" s="6"/>
@@ -3094,7 +3246,7 @@
       <c r="Y68" s="4"/>
       <c r="Z68" s="5"/>
     </row>
-    <row r="69" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A69" s="6"/>
       <c r="B69" s="6"/>
       <c r="C69" s="6"/>
@@ -3122,7 +3274,7 @@
       <c r="Y69" s="4"/>
       <c r="Z69" s="5"/>
     </row>
-    <row r="70" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A70" s="6"/>
       <c r="B70" s="6"/>
       <c r="C70" s="6"/>
@@ -3150,7 +3302,7 @@
       <c r="Y70" s="4"/>
       <c r="Z70" s="5"/>
     </row>
-    <row r="71" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A71" s="6"/>
       <c r="B71" s="6"/>
       <c r="C71" s="6"/>
@@ -3178,7 +3330,7 @@
       <c r="Y71" s="4"/>
       <c r="Z71" s="5"/>
     </row>
-    <row r="72" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A72" s="6"/>
       <c r="B72" s="6"/>
       <c r="C72" s="6"/>
@@ -3206,7 +3358,7 @@
       <c r="Y72" s="4"/>
       <c r="Z72" s="5"/>
     </row>
-    <row r="73" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A73" s="6"/>
       <c r="B73" s="6"/>
       <c r="C73" s="6"/>
@@ -3234,7 +3386,7 @@
       <c r="Y73" s="4"/>
       <c r="Z73" s="5"/>
     </row>
-    <row r="74" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A74" s="6"/>
       <c r="B74" s="6"/>
       <c r="C74" s="6"/>
@@ -3262,7 +3414,7 @@
       <c r="Y74" s="4"/>
       <c r="Z74" s="5"/>
     </row>
-    <row r="75" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A75" s="6"/>
       <c r="B75" s="6"/>
       <c r="C75" s="6"/>
@@ -3290,7 +3442,7 @@
       <c r="Y75" s="4"/>
       <c r="Z75" s="5"/>
     </row>
-    <row r="76" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A76" s="6"/>
       <c r="B76" s="6"/>
       <c r="C76" s="6"/>
@@ -3318,7 +3470,7 @@
       <c r="Y76" s="4"/>
       <c r="Z76" s="5"/>
     </row>
-    <row r="77" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A77" s="6"/>
       <c r="B77" s="6"/>
       <c r="C77" s="6"/>
@@ -3346,7 +3498,7 @@
       <c r="Y77" s="4"/>
       <c r="Z77" s="5"/>
     </row>
-    <row r="78" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A78" s="6"/>
       <c r="B78" s="6"/>
       <c r="C78" s="6"/>
@@ -3374,7 +3526,7 @@
       <c r="Y78" s="4"/>
       <c r="Z78" s="5"/>
     </row>
-    <row r="79" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A79" s="6"/>
       <c r="B79" s="6"/>
       <c r="C79" s="6"/>
@@ -3402,7 +3554,7 @@
       <c r="Y79" s="4"/>
       <c r="Z79" s="5"/>
     </row>
-    <row r="80" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A80" s="6"/>
       <c r="B80" s="6"/>
       <c r="C80" s="6"/>
@@ -3430,7 +3582,7 @@
       <c r="Y80" s="4"/>
       <c r="Z80" s="5"/>
     </row>
-    <row r="81" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A81" s="6"/>
       <c r="B81" s="6"/>
       <c r="C81" s="6"/>
@@ -3458,7 +3610,7 @@
       <c r="Y81" s="4"/>
       <c r="Z81" s="5"/>
     </row>
-    <row r="82" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A82" s="6"/>
       <c r="B82" s="6"/>
       <c r="C82" s="6"/>
@@ -3486,7 +3638,7 @@
       <c r="Y82" s="4"/>
       <c r="Z82" s="5"/>
     </row>
-    <row r="83" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A83" s="6"/>
       <c r="B83" s="6"/>
       <c r="C83" s="6"/>
@@ -3514,7 +3666,7 @@
       <c r="Y83" s="4"/>
       <c r="Z83" s="5"/>
     </row>
-    <row r="84" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A84" s="6"/>
       <c r="B84" s="6"/>
       <c r="C84" s="6"/>
@@ -3542,7 +3694,7 @@
       <c r="Y84" s="4"/>
       <c r="Z84" s="5"/>
     </row>
-    <row r="85" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A85" s="6"/>
       <c r="B85" s="6"/>
       <c r="C85" s="6"/>
@@ -3570,7 +3722,7 @@
       <c r="Y85" s="4"/>
       <c r="Z85" s="5"/>
     </row>
-    <row r="86" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A86" s="6"/>
       <c r="B86" s="6"/>
       <c r="C86" s="6"/>
@@ -3598,7 +3750,7 @@
       <c r="Y86" s="4"/>
       <c r="Z86" s="5"/>
     </row>
-    <row r="87" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A87" s="6"/>
       <c r="B87" s="6"/>
       <c r="C87" s="6"/>
@@ -3626,7 +3778,7 @@
       <c r="Y87" s="4"/>
       <c r="Z87" s="5"/>
     </row>
-    <row r="88" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A88" s="6"/>
       <c r="B88" s="6"/>
       <c r="C88" s="6"/>
@@ -3654,7 +3806,7 @@
       <c r="Y88" s="4"/>
       <c r="Z88" s="5"/>
     </row>
-    <row r="89" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A89" s="6"/>
       <c r="B89" s="6"/>
       <c r="C89" s="6"/>
@@ -3682,7 +3834,7 @@
       <c r="Y89" s="4"/>
       <c r="Z89" s="5"/>
     </row>
-    <row r="90" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A90" s="6"/>
       <c r="B90" s="6"/>
       <c r="C90" s="6"/>
@@ -3710,7 +3862,7 @@
       <c r="Y90" s="4"/>
       <c r="Z90" s="5"/>
     </row>
-    <row r="91" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A91" s="6"/>
       <c r="B91" s="6"/>
       <c r="C91" s="6"/>
@@ -3738,7 +3890,7 @@
       <c r="Y91" s="4"/>
       <c r="Z91" s="5"/>
     </row>
-    <row r="92" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A92" s="6"/>
       <c r="B92" s="6"/>
       <c r="C92" s="6"/>
@@ -3766,7 +3918,7 @@
       <c r="Y92" s="4"/>
       <c r="Z92" s="5"/>
     </row>
-    <row r="93" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A93" s="6"/>
       <c r="B93" s="6"/>
       <c r="C93" s="6"/>
@@ -3794,7 +3946,7 @@
       <c r="Y93" s="4"/>
       <c r="Z93" s="5"/>
     </row>
-    <row r="94" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A94" s="6"/>
       <c r="B94" s="6"/>
       <c r="C94" s="6"/>
@@ -3822,7 +3974,7 @@
       <c r="Y94" s="4"/>
       <c r="Z94" s="5"/>
     </row>
-    <row r="95" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A95" s="6"/>
       <c r="B95" s="6"/>
       <c r="C95" s="6"/>
@@ -3850,7 +4002,7 @@
       <c r="Y95" s="4"/>
       <c r="Z95" s="5"/>
     </row>
-    <row r="96" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A96" s="6"/>
       <c r="B96" s="6"/>
       <c r="C96" s="6"/>
@@ -3878,7 +4030,7 @@
       <c r="Y96" s="4"/>
       <c r="Z96" s="5"/>
     </row>
-    <row r="97" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A97" s="6"/>
       <c r="B97" s="6"/>
       <c r="C97" s="6"/>
@@ -3906,7 +4058,7 @@
       <c r="Y97" s="4"/>
       <c r="Z97" s="5"/>
     </row>
-    <row r="98" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A98" s="6"/>
       <c r="B98" s="6"/>
       <c r="C98" s="6"/>
@@ -3934,7 +4086,7 @@
       <c r="Y98" s="4"/>
       <c r="Z98" s="5"/>
     </row>
-    <row r="99" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A99" s="6"/>
       <c r="B99" s="6"/>
       <c r="C99" s="6"/>
@@ -3962,7 +4114,7 @@
       <c r="Y99" s="4"/>
       <c r="Z99" s="5"/>
     </row>
-    <row r="100" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A100" s="6"/>
       <c r="B100" s="6"/>
       <c r="C100" s="6"/>
@@ -3990,7 +4142,7 @@
       <c r="Y100" s="4"/>
       <c r="Z100" s="5"/>
     </row>
-    <row r="101" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A101" s="6"/>
       <c r="B101" s="6"/>
       <c r="C101" s="6"/>
@@ -4018,7 +4170,7 @@
       <c r="Y101" s="4"/>
       <c r="Z101" s="5"/>
     </row>
-    <row r="102" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A102" s="6"/>
       <c r="B102" s="6"/>
       <c r="C102" s="6"/>
@@ -4046,7 +4198,7 @@
       <c r="Y102" s="4"/>
       <c r="Z102" s="5"/>
     </row>
-    <row r="103" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A103" s="6"/>
       <c r="B103" s="6"/>
       <c r="C103" s="6"/>
@@ -4074,7 +4226,7 @@
       <c r="Y103" s="4"/>
       <c r="Z103" s="5"/>
     </row>
-    <row r="104" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A104" s="6"/>
       <c r="B104" s="6"/>
       <c r="C104" s="6"/>
@@ -4102,7 +4254,7 @@
       <c r="Y104" s="4"/>
       <c r="Z104" s="5"/>
     </row>
-    <row r="105" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A105" s="6"/>
       <c r="B105" s="6"/>
       <c r="C105" s="6"/>
@@ -4130,7 +4282,7 @@
       <c r="Y105" s="4"/>
       <c r="Z105" s="5"/>
     </row>
-    <row r="106" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A106" s="6"/>
       <c r="B106" s="6"/>
       <c r="C106" s="6"/>
@@ -4158,7 +4310,7 @@
       <c r="Y106" s="4"/>
       <c r="Z106" s="5"/>
     </row>
-    <row r="107" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A107" s="6"/>
       <c r="B107" s="6"/>
       <c r="C107" s="6"/>
@@ -4186,7 +4338,7 @@
       <c r="Y107" s="4"/>
       <c r="Z107" s="5"/>
     </row>
-    <row r="108" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A108" s="6"/>
       <c r="B108" s="6"/>
       <c r="C108" s="6"/>
@@ -4214,7 +4366,7 @@
       <c r="Y108" s="4"/>
       <c r="Z108" s="5"/>
     </row>
-    <row r="109" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A109" s="6"/>
       <c r="B109" s="6"/>
       <c r="C109" s="6"/>
@@ -4242,7 +4394,7 @@
       <c r="Y109" s="4"/>
       <c r="Z109" s="5"/>
     </row>
-    <row r="110" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A110" s="6"/>
       <c r="B110" s="6"/>
       <c r="C110" s="6"/>
@@ -4270,7 +4422,7 @@
       <c r="Y110" s="4"/>
       <c r="Z110" s="5"/>
     </row>
-    <row r="111" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A111" s="6"/>
       <c r="B111" s="6"/>
       <c r="C111" s="6"/>
@@ -4298,7 +4450,7 @@
       <c r="Y111" s="4"/>
       <c r="Z111" s="5"/>
     </row>
-    <row r="112" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A112" s="6"/>
       <c r="B112" s="6"/>
       <c r="C112" s="6"/>
@@ -4326,7 +4478,7 @@
       <c r="Y112" s="4"/>
       <c r="Z112" s="5"/>
     </row>
-    <row r="113" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A113" s="6"/>
       <c r="B113" s="6"/>
       <c r="C113" s="6"/>
@@ -4354,7 +4506,7 @@
       <c r="Y113" s="4"/>
       <c r="Z113" s="5"/>
     </row>
-    <row r="114" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A114" s="6"/>
       <c r="B114" s="6"/>
       <c r="C114" s="6"/>
@@ -4382,7 +4534,7 @@
       <c r="Y114" s="4"/>
       <c r="Z114" s="5"/>
     </row>
-    <row r="115" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A115" s="6"/>
       <c r="B115" s="6"/>
       <c r="C115" s="6"/>
@@ -4410,7 +4562,7 @@
       <c r="Y115" s="4"/>
       <c r="Z115" s="5"/>
     </row>
-    <row r="116" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A116" s="6"/>
       <c r="B116" s="6"/>
       <c r="C116" s="6"/>
@@ -4438,7 +4590,7 @@
       <c r="Y116" s="4"/>
       <c r="Z116" s="5"/>
     </row>
-    <row r="117" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A117" s="6"/>
       <c r="B117" s="6"/>
       <c r="C117" s="6"/>
@@ -4466,7 +4618,7 @@
       <c r="Y117" s="4"/>
       <c r="Z117" s="5"/>
     </row>
-    <row r="118" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A118" s="6"/>
       <c r="B118" s="6"/>
       <c r="C118" s="6"/>
@@ -4494,7 +4646,7 @@
       <c r="Y118" s="4"/>
       <c r="Z118" s="5"/>
     </row>
-    <row r="119" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A119" s="6"/>
       <c r="B119" s="6"/>
       <c r="C119" s="6"/>
@@ -4522,7 +4674,7 @@
       <c r="Y119" s="4"/>
       <c r="Z119" s="5"/>
     </row>
-    <row r="120" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A120" s="6"/>
       <c r="B120" s="6"/>
       <c r="C120" s="6"/>
@@ -4550,7 +4702,7 @@
       <c r="Y120" s="4"/>
       <c r="Z120" s="5"/>
     </row>
-    <row r="121" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A121" s="6"/>
       <c r="B121" s="6"/>
       <c r="C121" s="6"/>
@@ -4578,7 +4730,7 @@
       <c r="Y121" s="4"/>
       <c r="Z121" s="5"/>
     </row>
-    <row r="122" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A122" s="6"/>
       <c r="B122" s="6"/>
       <c r="C122" s="6"/>
@@ -4606,7 +4758,7 @@
       <c r="Y122" s="4"/>
       <c r="Z122" s="5"/>
     </row>
-    <row r="123" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A123" s="6"/>
       <c r="B123" s="6"/>
       <c r="C123" s="6"/>
@@ -4634,7 +4786,7 @@
       <c r="Y123" s="4"/>
       <c r="Z123" s="5"/>
     </row>
-    <row r="124" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A124" s="6"/>
       <c r="B124" s="6"/>
       <c r="C124" s="6"/>
@@ -4662,7 +4814,7 @@
       <c r="Y124" s="4"/>
       <c r="Z124" s="5"/>
     </row>
-    <row r="125" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A125" s="6"/>
       <c r="B125" s="6"/>
       <c r="C125" s="6"/>
@@ -4690,7 +4842,7 @@
       <c r="Y125" s="4"/>
       <c r="Z125" s="5"/>
     </row>
-    <row r="126" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A126" s="6"/>
       <c r="B126" s="6"/>
       <c r="C126" s="6"/>
@@ -4718,7 +4870,7 @@
       <c r="Y126" s="4"/>
       <c r="Z126" s="5"/>
     </row>
-    <row r="127" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A127" s="6"/>
       <c r="B127" s="6"/>
       <c r="C127" s="6"/>
@@ -4746,7 +4898,7 @@
       <c r="Y127" s="4"/>
       <c r="Z127" s="5"/>
     </row>
-    <row r="128" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A128" s="6"/>
       <c r="B128" s="6"/>
       <c r="C128" s="6"/>
@@ -4774,7 +4926,7 @@
       <c r="Y128" s="4"/>
       <c r="Z128" s="5"/>
     </row>
-    <row r="129" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A129" s="6"/>
       <c r="B129" s="6"/>
       <c r="C129" s="6"/>
@@ -4802,7 +4954,7 @@
       <c r="Y129" s="4"/>
       <c r="Z129" s="5"/>
     </row>
-    <row r="130" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A130" s="6"/>
       <c r="B130" s="6"/>
       <c r="C130" s="6"/>
@@ -4830,7 +4982,7 @@
       <c r="Y130" s="4"/>
       <c r="Z130" s="5"/>
     </row>
-    <row r="131" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A131" s="6"/>
       <c r="B131" s="6"/>
       <c r="C131" s="6"/>
@@ -4858,7 +5010,7 @@
       <c r="Y131" s="4"/>
       <c r="Z131" s="5"/>
     </row>
-    <row r="132" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A132" s="6"/>
       <c r="B132" s="6"/>
       <c r="C132" s="6"/>
@@ -4886,7 +5038,7 @@
       <c r="Y132" s="4"/>
       <c r="Z132" s="5"/>
     </row>
-    <row r="133" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A133" s="6"/>
       <c r="B133" s="6"/>
       <c r="C133" s="6"/>
@@ -4914,7 +5066,7 @@
       <c r="Y133" s="4"/>
       <c r="Z133" s="5"/>
     </row>
-    <row r="134" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A134" s="6"/>
       <c r="B134" s="6"/>
       <c r="C134" s="6"/>
@@ -4942,7 +5094,7 @@
       <c r="Y134" s="4"/>
       <c r="Z134" s="5"/>
     </row>
-    <row r="135" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A135" s="6"/>
       <c r="B135" s="6"/>
       <c r="C135" s="6"/>
@@ -4970,7 +5122,7 @@
       <c r="Y135" s="4"/>
       <c r="Z135" s="5"/>
     </row>
-    <row r="136" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A136" s="6"/>
       <c r="B136" s="6"/>
       <c r="C136" s="6"/>
@@ -4998,7 +5150,7 @@
       <c r="Y136" s="4"/>
       <c r="Z136" s="5"/>
     </row>
-    <row r="137" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A137" s="6"/>
       <c r="B137" s="6"/>
       <c r="C137" s="6"/>
@@ -5026,7 +5178,7 @@
       <c r="Y137" s="4"/>
       <c r="Z137" s="5"/>
     </row>
-    <row r="138" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A138" s="6"/>
       <c r="B138" s="6"/>
       <c r="C138" s="6"/>
@@ -5054,7 +5206,7 @@
       <c r="Y138" s="4"/>
       <c r="Z138" s="5"/>
     </row>
-    <row r="139" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A139" s="6"/>
       <c r="B139" s="6"/>
       <c r="C139" s="6"/>
@@ -5082,7 +5234,7 @@
       <c r="Y139" s="4"/>
       <c r="Z139" s="5"/>
     </row>
-    <row r="140" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A140" s="6"/>
       <c r="B140" s="6"/>
       <c r="C140" s="6"/>
@@ -5110,7 +5262,7 @@
       <c r="Y140" s="4"/>
       <c r="Z140" s="5"/>
     </row>
-    <row r="141" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A141" s="6"/>
       <c r="B141" s="6"/>
       <c r="C141" s="6"/>
@@ -5138,7 +5290,7 @@
       <c r="Y141" s="4"/>
       <c r="Z141" s="5"/>
     </row>
-    <row r="142" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A142" s="6"/>
       <c r="B142" s="6"/>
       <c r="C142" s="6"/>
@@ -5166,7 +5318,7 @@
       <c r="Y142" s="4"/>
       <c r="Z142" s="5"/>
     </row>
-    <row r="143" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A143" s="6"/>
       <c r="B143" s="6"/>
       <c r="C143" s="6"/>
@@ -5194,7 +5346,7 @@
       <c r="Y143" s="4"/>
       <c r="Z143" s="5"/>
     </row>
-    <row r="144" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A144" s="6"/>
       <c r="B144" s="6"/>
       <c r="C144" s="6"/>
@@ -5222,7 +5374,7 @@
       <c r="Y144" s="4"/>
       <c r="Z144" s="5"/>
     </row>
-    <row r="145" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A145" s="6"/>
       <c r="B145" s="6"/>
       <c r="C145" s="6"/>
@@ -5250,7 +5402,7 @@
       <c r="Y145" s="4"/>
       <c r="Z145" s="5"/>
     </row>
-    <row r="146" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A146" s="6"/>
       <c r="B146" s="6"/>
       <c r="C146" s="6"/>
@@ -5278,7 +5430,7 @@
       <c r="Y146" s="4"/>
       <c r="Z146" s="5"/>
     </row>
-    <row r="147" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A147" s="6"/>
       <c r="B147" s="6"/>
       <c r="C147" s="6"/>
@@ -5306,7 +5458,7 @@
       <c r="Y147" s="4"/>
       <c r="Z147" s="5"/>
     </row>
-    <row r="148" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A148" s="6"/>
       <c r="B148" s="6"/>
       <c r="C148" s="6"/>
@@ -5334,7 +5486,7 @@
       <c r="Y148" s="4"/>
       <c r="Z148" s="5"/>
     </row>
-    <row r="149" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A149" s="6"/>
       <c r="B149" s="6"/>
       <c r="C149" s="6"/>
@@ -5362,7 +5514,7 @@
       <c r="Y149" s="4"/>
       <c r="Z149" s="5"/>
     </row>
-    <row r="150" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A150" s="6"/>
       <c r="B150" s="6"/>
       <c r="C150" s="6"/>
@@ -5390,7 +5542,7 @@
       <c r="Y150" s="4"/>
       <c r="Z150" s="5"/>
     </row>
-    <row r="151" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A151" s="6"/>
       <c r="B151" s="6"/>
       <c r="C151" s="6"/>
@@ -5418,7 +5570,7 @@
       <c r="Y151" s="4"/>
       <c r="Z151" s="5"/>
     </row>
-    <row r="152" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A152" s="6"/>
       <c r="B152" s="6"/>
       <c r="C152" s="6"/>
@@ -5446,7 +5598,7 @@
       <c r="Y152" s="4"/>
       <c r="Z152" s="5"/>
     </row>
-    <row r="153" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A153" s="6"/>
       <c r="B153" s="6"/>
       <c r="C153" s="6"/>
@@ -5474,7 +5626,7 @@
       <c r="Y153" s="4"/>
       <c r="Z153" s="5"/>
     </row>
-    <row r="154" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A154" s="6"/>
       <c r="B154" s="6"/>
       <c r="C154" s="6"/>
@@ -5502,7 +5654,7 @@
       <c r="Y154" s="4"/>
       <c r="Z154" s="5"/>
     </row>
-    <row r="155" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A155" s="6"/>
       <c r="B155" s="6"/>
       <c r="C155" s="6"/>
@@ -5530,7 +5682,7 @@
       <c r="Y155" s="4"/>
       <c r="Z155" s="5"/>
     </row>
-    <row r="156" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A156" s="6"/>
       <c r="B156" s="6"/>
       <c r="C156" s="6"/>
@@ -5558,7 +5710,7 @@
       <c r="Y156" s="4"/>
       <c r="Z156" s="5"/>
     </row>
-    <row r="157" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A157" s="6"/>
       <c r="B157" s="6"/>
       <c r="C157" s="6"/>
@@ -5586,7 +5738,7 @@
       <c r="Y157" s="4"/>
       <c r="Z157" s="5"/>
     </row>
-    <row r="158" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A158" s="6"/>
       <c r="B158" s="6"/>
       <c r="C158" s="6"/>
@@ -5614,7 +5766,7 @@
       <c r="Y158" s="4"/>
       <c r="Z158" s="5"/>
     </row>
-    <row r="159" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A159" s="6"/>
       <c r="B159" s="6"/>
       <c r="C159" s="6"/>
@@ -5642,7 +5794,7 @@
       <c r="Y159" s="4"/>
       <c r="Z159" s="5"/>
     </row>
-    <row r="160" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A160" s="6"/>
       <c r="B160" s="6"/>
       <c r="C160" s="6"/>
@@ -5670,7 +5822,7 @@
       <c r="Y160" s="4"/>
       <c r="Z160" s="5"/>
     </row>
-    <row r="161" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A161" s="6"/>
       <c r="B161" s="6"/>
       <c r="C161" s="6"/>
@@ -5698,7 +5850,7 @@
       <c r="Y161" s="4"/>
       <c r="Z161" s="5"/>
     </row>
-    <row r="162" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A162" s="6"/>
       <c r="B162" s="6"/>
       <c r="C162" s="6"/>
@@ -5726,7 +5878,7 @@
       <c r="Y162" s="4"/>
       <c r="Z162" s="5"/>
     </row>
-    <row r="163" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A163" s="6"/>
       <c r="B163" s="6"/>
       <c r="C163" s="6"/>
@@ -5754,7 +5906,7 @@
       <c r="Y163" s="4"/>
       <c r="Z163" s="5"/>
     </row>
-    <row r="164" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A164" s="6"/>
       <c r="B164" s="6"/>
       <c r="C164" s="6"/>
@@ -5782,7 +5934,7 @@
       <c r="Y164" s="4"/>
       <c r="Z164" s="5"/>
     </row>
-    <row r="165" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A165" s="6"/>
       <c r="B165" s="6"/>
       <c r="C165" s="6"/>
@@ -5810,7 +5962,7 @@
       <c r="Y165" s="4"/>
       <c r="Z165" s="5"/>
     </row>
-    <row r="166" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A166" s="6"/>
       <c r="B166" s="6"/>
       <c r="C166" s="6"/>
@@ -5838,7 +5990,7 @@
       <c r="Y166" s="4"/>
       <c r="Z166" s="5"/>
     </row>
-    <row r="167" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A167" s="6"/>
       <c r="B167" s="6"/>
       <c r="C167" s="6"/>
@@ -5866,7 +6018,7 @@
       <c r="Y167" s="4"/>
       <c r="Z167" s="5"/>
     </row>
-    <row r="168" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A168" s="6"/>
       <c r="B168" s="6"/>
       <c r="C168" s="6"/>
@@ -5894,7 +6046,7 @@
       <c r="Y168" s="4"/>
       <c r="Z168" s="5"/>
     </row>
-    <row r="169" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A169" s="6"/>
       <c r="B169" s="6"/>
       <c r="C169" s="6"/>
@@ -5922,7 +6074,7 @@
       <c r="Y169" s="4"/>
       <c r="Z169" s="5"/>
     </row>
-    <row r="170" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A170" s="6"/>
       <c r="B170" s="6"/>
       <c r="C170" s="6"/>
@@ -5950,7 +6102,7 @@
       <c r="Y170" s="4"/>
       <c r="Z170" s="5"/>
     </row>
-    <row r="171" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A171" s="6"/>
       <c r="B171" s="6"/>
       <c r="C171" s="6"/>
@@ -5978,7 +6130,7 @@
       <c r="Y171" s="4"/>
       <c r="Z171" s="5"/>
     </row>
-    <row r="172" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A172" s="6"/>
       <c r="B172" s="6"/>
       <c r="C172" s="6"/>
@@ -6006,7 +6158,7 @@
       <c r="Y172" s="4"/>
       <c r="Z172" s="5"/>
     </row>
-    <row r="173" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A173" s="6"/>
       <c r="B173" s="6"/>
       <c r="C173" s="6"/>
@@ -6034,7 +6186,7 @@
       <c r="Y173" s="4"/>
       <c r="Z173" s="5"/>
     </row>
-    <row r="174" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A174" s="6"/>
       <c r="B174" s="6"/>
       <c r="C174" s="6"/>
@@ -6062,7 +6214,7 @@
       <c r="Y174" s="4"/>
       <c r="Z174" s="5"/>
     </row>
-    <row r="175" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A175" s="6"/>
       <c r="B175" s="6"/>
       <c r="C175" s="6"/>
@@ -6090,7 +6242,7 @@
       <c r="Y175" s="4"/>
       <c r="Z175" s="5"/>
     </row>
-    <row r="176" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A176" s="6"/>
       <c r="B176" s="6"/>
       <c r="C176" s="6"/>
@@ -6118,7 +6270,7 @@
       <c r="Y176" s="4"/>
       <c r="Z176" s="5"/>
     </row>
-    <row r="177" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A177" s="6"/>
       <c r="B177" s="6"/>
       <c r="C177" s="6"/>
@@ -6146,7 +6298,7 @@
       <c r="Y177" s="4"/>
       <c r="Z177" s="5"/>
     </row>
-    <row r="178" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A178" s="6"/>
       <c r="B178" s="6"/>
       <c r="C178" s="6"/>
@@ -6174,7 +6326,7 @@
       <c r="Y178" s="4"/>
       <c r="Z178" s="5"/>
     </row>
-    <row r="179" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A179" s="6"/>
       <c r="B179" s="6"/>
       <c r="C179" s="6"/>
@@ -6202,7 +6354,7 @@
       <c r="Y179" s="4"/>
       <c r="Z179" s="5"/>
     </row>
-    <row r="180" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A180" s="6"/>
       <c r="B180" s="6"/>
       <c r="C180" s="6"/>
@@ -6230,7 +6382,7 @@
       <c r="Y180" s="4"/>
       <c r="Z180" s="5"/>
     </row>
-    <row r="181" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A181" s="6"/>
       <c r="B181" s="6"/>
       <c r="C181" s="6"/>
@@ -6258,7 +6410,7 @@
       <c r="Y181" s="4"/>
       <c r="Z181" s="5"/>
     </row>
-    <row r="182" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A182" s="6"/>
       <c r="B182" s="6"/>
       <c r="C182" s="6"/>
@@ -6286,7 +6438,7 @@
       <c r="Y182" s="4"/>
       <c r="Z182" s="5"/>
     </row>
-    <row r="183" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A183" s="6"/>
       <c r="B183" s="6"/>
       <c r="C183" s="6"/>
@@ -6314,7 +6466,7 @@
       <c r="Y183" s="4"/>
       <c r="Z183" s="5"/>
     </row>
-    <row r="184" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A184" s="6"/>
       <c r="B184" s="6"/>
       <c r="C184" s="6"/>
@@ -6342,7 +6494,7 @@
       <c r="Y184" s="4"/>
       <c r="Z184" s="5"/>
     </row>
-    <row r="185" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A185" s="6"/>
       <c r="B185" s="6"/>
       <c r="C185" s="6"/>
@@ -6370,7 +6522,7 @@
       <c r="Y185" s="4"/>
       <c r="Z185" s="5"/>
     </row>
-    <row r="186" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A186" s="6"/>
       <c r="B186" s="6"/>
       <c r="C186" s="6"/>
@@ -6398,7 +6550,7 @@
       <c r="Y186" s="4"/>
       <c r="Z186" s="5"/>
     </row>
-    <row r="187" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A187" s="6"/>
       <c r="B187" s="6"/>
       <c r="C187" s="6"/>
@@ -6426,7 +6578,7 @@
       <c r="Y187" s="4"/>
       <c r="Z187" s="5"/>
     </row>
-    <row r="188" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A188" s="6"/>
       <c r="B188" s="6"/>
       <c r="C188" s="6"/>
@@ -6454,7 +6606,7 @@
       <c r="Y188" s="4"/>
       <c r="Z188" s="5"/>
     </row>
-    <row r="189" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A189" s="6"/>
       <c r="B189" s="6"/>
       <c r="C189" s="6"/>
@@ -6482,7 +6634,7 @@
       <c r="Y189" s="4"/>
       <c r="Z189" s="5"/>
     </row>
-    <row r="190" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A190" s="6"/>
       <c r="B190" s="6"/>
       <c r="C190" s="6"/>
@@ -6510,7 +6662,7 @@
       <c r="Y190" s="4"/>
       <c r="Z190" s="5"/>
     </row>
-    <row r="191" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A191" s="6"/>
       <c r="B191" s="6"/>
       <c r="C191" s="6"/>
@@ -6538,7 +6690,7 @@
       <c r="Y191" s="4"/>
       <c r="Z191" s="5"/>
     </row>
-    <row r="192" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A192" s="6"/>
       <c r="B192" s="6"/>
       <c r="C192" s="6"/>
@@ -6566,7 +6718,7 @@
       <c r="Y192" s="4"/>
       <c r="Z192" s="5"/>
     </row>
-    <row r="193" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A193" s="6"/>
       <c r="B193" s="6"/>
       <c r="C193" s="6"/>
@@ -6594,7 +6746,7 @@
       <c r="Y193" s="4"/>
       <c r="Z193" s="5"/>
     </row>
-    <row r="194" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A194" s="6"/>
       <c r="B194" s="6"/>
       <c r="C194" s="6"/>
@@ -6622,7 +6774,7 @@
       <c r="Y194" s="4"/>
       <c r="Z194" s="5"/>
     </row>
-    <row r="195" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A195" s="6"/>
       <c r="B195" s="6"/>
       <c r="C195" s="6"/>
@@ -6650,7 +6802,7 @@
       <c r="Y195" s="4"/>
       <c r="Z195" s="5"/>
     </row>
-    <row r="196" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A196" s="6"/>
       <c r="B196" s="6"/>
       <c r="C196" s="6"/>
@@ -6678,7 +6830,7 @@
       <c r="Y196" s="4"/>
       <c r="Z196" s="5"/>
     </row>
-    <row r="197" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A197" s="6"/>
       <c r="B197" s="6"/>
       <c r="C197" s="6"/>
@@ -6706,7 +6858,7 @@
       <c r="Y197" s="4"/>
       <c r="Z197" s="5"/>
     </row>
-    <row r="198" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A198" s="6"/>
       <c r="B198" s="6"/>
       <c r="C198" s="6"/>
@@ -6734,7 +6886,7 @@
       <c r="Y198" s="4"/>
       <c r="Z198" s="5"/>
     </row>
-    <row r="199" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A199" s="6"/>
       <c r="B199" s="6"/>
       <c r="C199" s="6"/>
@@ -6762,7 +6914,7 @@
       <c r="Y199" s="4"/>
       <c r="Z199" s="5"/>
     </row>
-    <row r="200" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A200" s="6"/>
       <c r="B200" s="6"/>
       <c r="C200" s="6"/>
@@ -6790,7 +6942,7 @@
       <c r="Y200" s="4"/>
       <c r="Z200" s="5"/>
     </row>
-    <row r="201" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A201" s="6"/>
       <c r="B201" s="6"/>
       <c r="C201" s="6"/>
@@ -6818,7 +6970,7 @@
       <c r="Y201" s="4"/>
       <c r="Z201" s="5"/>
     </row>
-    <row r="202" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A202" s="6"/>
       <c r="B202" s="6"/>
       <c r="C202" s="6"/>
@@ -6846,7 +6998,7 @@
       <c r="Y202" s="4"/>
       <c r="Z202" s="5"/>
     </row>
-    <row r="203" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A203" s="6"/>
       <c r="B203" s="6"/>
       <c r="C203" s="6"/>
@@ -6874,7 +7026,7 @@
       <c r="Y203" s="4"/>
       <c r="Z203" s="5"/>
     </row>
-    <row r="204" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A204" s="6"/>
       <c r="B204" s="6"/>
       <c r="C204" s="6"/>
@@ -6902,7 +7054,7 @@
       <c r="Y204" s="4"/>
       <c r="Z204" s="5"/>
     </row>
-    <row r="205" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A205" s="6"/>
       <c r="B205" s="6"/>
       <c r="C205" s="6"/>
@@ -6930,7 +7082,7 @@
       <c r="Y205" s="4"/>
       <c r="Z205" s="5"/>
     </row>
-    <row r="206" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A206" s="6"/>
       <c r="B206" s="6"/>
       <c r="C206" s="6"/>
@@ -6958,7 +7110,7 @@
       <c r="Y206" s="4"/>
       <c r="Z206" s="5"/>
     </row>
-    <row r="207" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A207" s="6"/>
       <c r="B207" s="6"/>
       <c r="C207" s="6"/>
@@ -6986,7 +7138,7 @@
       <c r="Y207" s="4"/>
       <c r="Z207" s="5"/>
     </row>
-    <row r="208" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A208" s="6"/>
       <c r="B208" s="6"/>
       <c r="C208" s="6"/>
@@ -7014,7 +7166,7 @@
       <c r="Y208" s="4"/>
       <c r="Z208" s="5"/>
     </row>
-    <row r="209" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A209" s="6"/>
       <c r="B209" s="6"/>
       <c r="C209" s="6"/>
@@ -7042,7 +7194,7 @@
       <c r="Y209" s="4"/>
       <c r="Z209" s="5"/>
     </row>
-    <row r="210" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A210" s="6"/>
       <c r="B210" s="6"/>
       <c r="C210" s="6"/>
@@ -7070,7 +7222,7 @@
       <c r="Y210" s="4"/>
       <c r="Z210" s="5"/>
     </row>
-    <row r="211" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A211" s="6"/>
       <c r="B211" s="6"/>
       <c r="C211" s="6"/>
@@ -7098,7 +7250,7 @@
       <c r="Y211" s="4"/>
       <c r="Z211" s="5"/>
     </row>
-    <row r="212" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A212" s="6"/>
       <c r="B212" s="6"/>
       <c r="C212" s="6"/>
@@ -7126,7 +7278,7 @@
       <c r="Y212" s="4"/>
       <c r="Z212" s="5"/>
     </row>
-    <row r="213" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A213" s="6"/>
       <c r="B213" s="6"/>
       <c r="C213" s="6"/>
@@ -7154,7 +7306,7 @@
       <c r="Y213" s="4"/>
       <c r="Z213" s="5"/>
     </row>
-    <row r="214" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A214" s="6"/>
       <c r="B214" s="6"/>
       <c r="C214" s="6"/>
@@ -7182,7 +7334,7 @@
       <c r="Y214" s="4"/>
       <c r="Z214" s="5"/>
     </row>
-    <row r="215" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A215" s="6"/>
       <c r="B215" s="6"/>
       <c r="C215" s="6"/>
@@ -7210,7 +7362,7 @@
       <c r="Y215" s="4"/>
       <c r="Z215" s="5"/>
     </row>
-    <row r="216" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A216" s="6"/>
       <c r="B216" s="6"/>
       <c r="C216" s="6"/>
@@ -7238,7 +7390,7 @@
       <c r="Y216" s="4"/>
       <c r="Z216" s="5"/>
     </row>
-    <row r="217" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A217" s="6"/>
       <c r="B217" s="6"/>
       <c r="C217" s="6"/>
@@ -7266,7 +7418,7 @@
       <c r="Y217" s="4"/>
       <c r="Z217" s="5"/>
     </row>
-    <row r="218" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A218" s="6"/>
       <c r="B218" s="6"/>
       <c r="C218" s="6"/>
@@ -7294,7 +7446,7 @@
       <c r="Y218" s="4"/>
       <c r="Z218" s="5"/>
     </row>
-    <row r="219" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="219" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A219" s="6"/>
       <c r="B219" s="6"/>
       <c r="C219" s="6"/>
@@ -7322,7 +7474,7 @@
       <c r="Y219" s="4"/>
       <c r="Z219" s="5"/>
     </row>
-    <row r="220" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A220" s="6"/>
       <c r="B220" s="6"/>
       <c r="C220" s="6"/>
@@ -7350,7 +7502,7 @@
       <c r="Y220" s="4"/>
       <c r="Z220" s="5"/>
     </row>
-    <row r="221" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="221" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A221" s="6"/>
       <c r="B221" s="6"/>
       <c r="C221" s="6"/>
@@ -7378,7 +7530,7 @@
       <c r="Y221" s="4"/>
       <c r="Z221" s="5"/>
     </row>
-    <row r="222" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="222" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A222" s="6"/>
       <c r="B222" s="6"/>
       <c r="C222" s="6"/>
@@ -7406,7 +7558,7 @@
       <c r="Y222" s="4"/>
       <c r="Z222" s="5"/>
     </row>
-    <row r="223" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="223" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A223" s="6"/>
       <c r="B223" s="6"/>
       <c r="C223" s="6"/>
@@ -7434,7 +7586,7 @@
       <c r="Y223" s="4"/>
       <c r="Z223" s="5"/>
     </row>
-    <row r="224" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="224" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A224" s="6"/>
       <c r="B224" s="6"/>
       <c r="C224" s="6"/>
@@ -7462,7 +7614,7 @@
       <c r="Y224" s="4"/>
       <c r="Z224" s="5"/>
     </row>
-    <row r="225" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="225" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A225" s="6"/>
       <c r="B225" s="6"/>
       <c r="C225" s="6"/>
@@ -7490,7 +7642,7 @@
       <c r="Y225" s="4"/>
       <c r="Z225" s="5"/>
     </row>
-    <row r="226" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="226" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A226" s="6"/>
       <c r="B226" s="6"/>
       <c r="C226" s="6"/>
@@ -7518,7 +7670,7 @@
       <c r="Y226" s="4"/>
       <c r="Z226" s="5"/>
     </row>
-    <row r="227" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="227" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A227" s="6"/>
       <c r="B227" s="6"/>
       <c r="C227" s="6"/>
@@ -7546,7 +7698,7 @@
       <c r="Y227" s="4"/>
       <c r="Z227" s="5"/>
     </row>
-    <row r="228" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="228" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A228" s="6"/>
       <c r="B228" s="6"/>
       <c r="C228" s="6"/>
@@ -7574,7 +7726,7 @@
       <c r="Y228" s="4"/>
       <c r="Z228" s="5"/>
     </row>
-    <row r="229" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="229" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A229" s="6"/>
       <c r="B229" s="6"/>
       <c r="C229" s="6"/>
@@ -7602,7 +7754,7 @@
       <c r="Y229" s="4"/>
       <c r="Z229" s="5"/>
     </row>
-    <row r="230" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="230" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A230" s="6"/>
       <c r="B230" s="6"/>
       <c r="C230" s="6"/>
@@ -7630,7 +7782,7 @@
       <c r="Y230" s="4"/>
       <c r="Z230" s="5"/>
     </row>
-    <row r="231" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="231" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A231" s="6"/>
       <c r="B231" s="6"/>
       <c r="C231" s="6"/>
@@ -7658,7 +7810,7 @@
       <c r="Y231" s="4"/>
       <c r="Z231" s="5"/>
     </row>
-    <row r="232" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="232" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A232" s="6"/>
       <c r="B232" s="6"/>
       <c r="C232" s="6"/>
@@ -7686,7 +7838,7 @@
       <c r="Y232" s="4"/>
       <c r="Z232" s="5"/>
     </row>
-    <row r="233" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="233" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A233" s="6"/>
       <c r="B233" s="6"/>
       <c r="C233" s="6"/>
@@ -7714,7 +7866,7 @@
       <c r="Y233" s="4"/>
       <c r="Z233" s="5"/>
     </row>
-    <row r="234" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="234" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A234" s="6"/>
       <c r="B234" s="6"/>
       <c r="C234" s="6"/>
@@ -7742,7 +7894,7 @@
       <c r="Y234" s="4"/>
       <c r="Z234" s="5"/>
     </row>
-    <row r="235" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="235" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A235" s="6"/>
       <c r="B235" s="6"/>
       <c r="C235" s="6"/>
@@ -7770,7 +7922,7 @@
       <c r="Y235" s="4"/>
       <c r="Z235" s="5"/>
     </row>
-    <row r="236" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="236" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A236" s="6"/>
       <c r="B236" s="6"/>
       <c r="C236" s="6"/>
@@ -7798,7 +7950,7 @@
       <c r="Y236" s="4"/>
       <c r="Z236" s="5"/>
     </row>
-    <row r="237" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="237" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A237" s="6"/>
       <c r="B237" s="6"/>
       <c r="C237" s="6"/>
@@ -7826,7 +7978,7 @@
       <c r="Y237" s="4"/>
       <c r="Z237" s="5"/>
     </row>
-    <row r="238" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="238" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A238" s="6"/>
       <c r="B238" s="6"/>
       <c r="C238" s="6"/>
@@ -7854,7 +8006,7 @@
       <c r="Y238" s="4"/>
       <c r="Z238" s="5"/>
     </row>
-    <row r="239" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="239" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A239" s="6"/>
       <c r="B239" s="6"/>
       <c r="C239" s="6"/>
@@ -7882,7 +8034,7 @@
       <c r="Y239" s="4"/>
       <c r="Z239" s="5"/>
     </row>
-    <row r="240" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="240" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A240" s="6"/>
       <c r="B240" s="6"/>
       <c r="C240" s="6"/>
@@ -7910,7 +8062,7 @@
       <c r="Y240" s="4"/>
       <c r="Z240" s="5"/>
     </row>
-    <row r="241" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="241" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A241" s="6"/>
       <c r="B241" s="6"/>
       <c r="C241" s="6"/>
@@ -7938,7 +8090,7 @@
       <c r="Y241" s="4"/>
       <c r="Z241" s="5"/>
     </row>
-    <row r="242" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="242" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A242" s="6"/>
       <c r="B242" s="6"/>
       <c r="C242" s="6"/>
@@ -7966,7 +8118,7 @@
       <c r="Y242" s="4"/>
       <c r="Z242" s="5"/>
     </row>
-    <row r="243" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="243" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A243" s="6"/>
       <c r="B243" s="6"/>
       <c r="C243" s="6"/>
@@ -7994,7 +8146,7 @@
       <c r="Y243" s="4"/>
       <c r="Z243" s="5"/>
     </row>
-    <row r="244" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="244" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A244" s="6"/>
       <c r="B244" s="6"/>
       <c r="C244" s="6"/>
@@ -8022,7 +8174,7 @@
       <c r="Y244" s="4"/>
       <c r="Z244" s="5"/>
     </row>
-    <row r="245" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="245" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A245" s="6"/>
       <c r="B245" s="6"/>
       <c r="C245" s="6"/>
@@ -8050,7 +8202,7 @@
       <c r="Y245" s="4"/>
       <c r="Z245" s="5"/>
     </row>
-    <row r="246" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="246" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A246" s="6"/>
       <c r="B246" s="6"/>
       <c r="C246" s="6"/>
@@ -8078,7 +8230,7 @@
       <c r="Y246" s="4"/>
       <c r="Z246" s="5"/>
     </row>
-    <row r="247" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="247" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A247" s="6"/>
       <c r="B247" s="6"/>
       <c r="C247" s="6"/>
@@ -8106,7 +8258,7 @@
       <c r="Y247" s="4"/>
       <c r="Z247" s="5"/>
     </row>
-    <row r="248" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="248" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A248" s="6"/>
       <c r="B248" s="6"/>
       <c r="C248" s="6"/>
@@ -8134,7 +8286,7 @@
       <c r="Y248" s="4"/>
       <c r="Z248" s="5"/>
     </row>
-    <row r="249" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="249" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A249" s="6"/>
       <c r="B249" s="6"/>
       <c r="C249" s="6"/>
@@ -8162,7 +8314,7 @@
       <c r="Y249" s="4"/>
       <c r="Z249" s="5"/>
     </row>
-    <row r="250" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="250" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A250" s="6"/>
       <c r="B250" s="6"/>
       <c r="C250" s="6"/>
@@ -8190,7 +8342,7 @@
       <c r="Y250" s="4"/>
       <c r="Z250" s="5"/>
     </row>
-    <row r="251" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="251" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A251" s="6"/>
       <c r="B251" s="6"/>
       <c r="C251" s="6"/>
@@ -8218,7 +8370,7 @@
       <c r="Y251" s="4"/>
       <c r="Z251" s="5"/>
     </row>
-    <row r="252" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="252" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A252" s="6"/>
       <c r="B252" s="6"/>
       <c r="C252" s="6"/>
@@ -8246,7 +8398,7 @@
       <c r="Y252" s="4"/>
       <c r="Z252" s="5"/>
     </row>
-    <row r="253" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="253" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A253" s="6"/>
       <c r="B253" s="6"/>
       <c r="C253" s="6"/>
@@ -8274,7 +8426,7 @@
       <c r="Y253" s="4"/>
       <c r="Z253" s="5"/>
     </row>
-    <row r="254" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="254" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A254" s="6"/>
       <c r="B254" s="6"/>
       <c r="C254" s="6"/>
@@ -8302,7 +8454,7 @@
       <c r="Y254" s="4"/>
       <c r="Z254" s="5"/>
     </row>
-    <row r="255" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="255" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A255" s="6"/>
       <c r="B255" s="6"/>
       <c r="C255" s="6"/>
@@ -8330,7 +8482,7 @@
       <c r="Y255" s="4"/>
       <c r="Z255" s="5"/>
     </row>
-    <row r="256" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="256" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A256" s="6"/>
       <c r="B256" s="6"/>
       <c r="C256" s="6"/>
@@ -8358,7 +8510,7 @@
       <c r="Y256" s="4"/>
       <c r="Z256" s="5"/>
     </row>
-    <row r="257" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="257" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A257" s="6"/>
       <c r="B257" s="6"/>
       <c r="C257" s="6"/>
@@ -8386,7 +8538,7 @@
       <c r="Y257" s="4"/>
       <c r="Z257" s="5"/>
     </row>
-    <row r="258" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="258" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A258" s="6"/>
       <c r="B258" s="6"/>
       <c r="C258" s="6"/>
@@ -8414,7 +8566,7 @@
       <c r="Y258" s="4"/>
       <c r="Z258" s="5"/>
     </row>
-    <row r="259" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="259" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A259" s="6"/>
       <c r="B259" s="6"/>
       <c r="C259" s="6"/>
@@ -8442,7 +8594,7 @@
       <c r="Y259" s="4"/>
       <c r="Z259" s="5"/>
     </row>
-    <row r="260" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="260" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A260" s="6"/>
       <c r="B260" s="6"/>
       <c r="C260" s="6"/>
@@ -8470,7 +8622,7 @@
       <c r="Y260" s="4"/>
       <c r="Z260" s="5"/>
     </row>
-    <row r="261" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="261" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A261" s="6"/>
       <c r="B261" s="6"/>
       <c r="C261" s="6"/>
@@ -8498,7 +8650,7 @@
       <c r="Y261" s="4"/>
       <c r="Z261" s="5"/>
     </row>
-    <row r="262" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="262" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A262" s="6"/>
       <c r="B262" s="6"/>
       <c r="C262" s="6"/>
@@ -8526,7 +8678,7 @@
       <c r="Y262" s="4"/>
       <c r="Z262" s="5"/>
     </row>
-    <row r="263" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="263" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A263" s="6"/>
       <c r="B263" s="6"/>
       <c r="C263" s="6"/>
@@ -8554,7 +8706,7 @@
       <c r="Y263" s="4"/>
       <c r="Z263" s="5"/>
     </row>
-    <row r="264" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="264" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A264" s="6"/>
       <c r="B264" s="6"/>
       <c r="C264" s="6"/>
@@ -8582,7 +8734,7 @@
       <c r="Y264" s="4"/>
       <c r="Z264" s="5"/>
     </row>
-    <row r="265" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="265" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A265" s="6"/>
       <c r="B265" s="6"/>
       <c r="C265" s="6"/>
@@ -8610,7 +8762,7 @@
       <c r="Y265" s="4"/>
       <c r="Z265" s="5"/>
     </row>
-    <row r="266" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="266" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A266" s="6"/>
       <c r="B266" s="6"/>
       <c r="C266" s="6"/>
@@ -8638,7 +8790,7 @@
       <c r="Y266" s="4"/>
       <c r="Z266" s="5"/>
     </row>
-    <row r="267" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="267" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A267" s="6"/>
       <c r="B267" s="6"/>
       <c r="C267" s="6"/>
@@ -8666,7 +8818,7 @@
       <c r="Y267" s="4"/>
       <c r="Z267" s="5"/>
     </row>
-    <row r="268" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="268" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A268" s="6"/>
       <c r="B268" s="6"/>
       <c r="C268" s="6"/>
@@ -8694,7 +8846,7 @@
       <c r="Y268" s="4"/>
       <c r="Z268" s="5"/>
     </row>
-    <row r="269" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="269" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A269" s="6"/>
       <c r="B269" s="6"/>
       <c r="C269" s="6"/>
@@ -8722,7 +8874,7 @@
       <c r="Y269" s="4"/>
       <c r="Z269" s="5"/>
     </row>
-    <row r="270" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="270" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A270" s="6"/>
       <c r="B270" s="6"/>
       <c r="C270" s="6"/>
@@ -8750,7 +8902,7 @@
       <c r="Y270" s="4"/>
       <c r="Z270" s="5"/>
     </row>
-    <row r="271" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="271" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A271" s="6"/>
       <c r="B271" s="6"/>
       <c r="C271" s="6"/>
@@ -8778,7 +8930,7 @@
       <c r="Y271" s="4"/>
       <c r="Z271" s="5"/>
     </row>
-    <row r="272" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="272" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A272" s="6"/>
       <c r="B272" s="6"/>
       <c r="C272" s="6"/>
@@ -8806,7 +8958,7 @@
       <c r="Y272" s="4"/>
       <c r="Z272" s="5"/>
     </row>
-    <row r="273" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="273" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A273" s="6"/>
       <c r="B273" s="6"/>
       <c r="C273" s="6"/>
@@ -8834,7 +8986,7 @@
       <c r="Y273" s="4"/>
       <c r="Z273" s="5"/>
     </row>
-    <row r="274" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="274" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A274" s="6"/>
       <c r="B274" s="6"/>
       <c r="C274" s="6"/>
@@ -8862,7 +9014,7 @@
       <c r="Y274" s="4"/>
       <c r="Z274" s="5"/>
     </row>
-    <row r="275" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="275" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A275" s="6"/>
       <c r="B275" s="6"/>
       <c r="C275" s="6"/>
@@ -8890,7 +9042,7 @@
       <c r="Y275" s="4"/>
       <c r="Z275" s="5"/>
     </row>
-    <row r="276" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="276" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A276" s="6"/>
       <c r="B276" s="6"/>
       <c r="C276" s="6"/>
@@ -8918,7 +9070,7 @@
       <c r="Y276" s="4"/>
       <c r="Z276" s="5"/>
     </row>
-    <row r="277" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="277" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A277" s="6"/>
       <c r="B277" s="6"/>
       <c r="C277" s="6"/>
@@ -8946,7 +9098,7 @@
       <c r="Y277" s="4"/>
       <c r="Z277" s="5"/>
     </row>
-    <row r="278" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="278" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A278" s="6"/>
       <c r="B278" s="6"/>
       <c r="C278" s="6"/>
@@ -8974,7 +9126,7 @@
       <c r="Y278" s="4"/>
       <c r="Z278" s="5"/>
     </row>
-    <row r="279" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="279" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A279" s="6"/>
       <c r="B279" s="6"/>
       <c r="C279" s="6"/>
@@ -9002,7 +9154,7 @@
       <c r="Y279" s="4"/>
       <c r="Z279" s="5"/>
     </row>
-    <row r="280" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="280" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A280" s="6"/>
       <c r="B280" s="6"/>
       <c r="C280" s="6"/>
@@ -9030,7 +9182,7 @@
       <c r="Y280" s="4"/>
       <c r="Z280" s="5"/>
     </row>
-    <row r="281" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="281" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A281" s="6"/>
       <c r="B281" s="6"/>
       <c r="C281" s="6"/>
@@ -9058,7 +9210,7 @@
       <c r="Y281" s="4"/>
       <c r="Z281" s="5"/>
     </row>
-    <row r="282" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="282" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A282" s="6"/>
       <c r="B282" s="6"/>
       <c r="C282" s="6"/>
@@ -9086,7 +9238,7 @@
       <c r="Y282" s="4"/>
       <c r="Z282" s="5"/>
     </row>
-    <row r="283" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="283" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A283" s="6"/>
       <c r="B283" s="6"/>
       <c r="C283" s="6"/>
@@ -9114,7 +9266,7 @@
       <c r="Y283" s="4"/>
       <c r="Z283" s="5"/>
     </row>
-    <row r="284" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="284" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A284" s="6"/>
       <c r="B284" s="6"/>
       <c r="C284" s="6"/>
@@ -9142,7 +9294,7 @@
       <c r="Y284" s="4"/>
       <c r="Z284" s="5"/>
     </row>
-    <row r="285" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="285" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A285" s="6"/>
       <c r="B285" s="6"/>
       <c r="C285" s="6"/>
@@ -9170,7 +9322,7 @@
       <c r="Y285" s="4"/>
       <c r="Z285" s="5"/>
     </row>
-    <row r="286" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="286" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A286" s="6"/>
       <c r="B286" s="6"/>
       <c r="C286" s="6"/>
@@ -9198,7 +9350,7 @@
       <c r="Y286" s="4"/>
       <c r="Z286" s="5"/>
     </row>
-    <row r="287" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="287" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A287" s="6"/>
       <c r="B287" s="6"/>
       <c r="C287" s="6"/>
@@ -9226,7 +9378,7 @@
       <c r="Y287" s="4"/>
       <c r="Z287" s="5"/>
     </row>
-    <row r="288" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="288" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A288" s="6"/>
       <c r="B288" s="6"/>
       <c r="C288" s="6"/>
@@ -9254,7 +9406,7 @@
       <c r="Y288" s="4"/>
       <c r="Z288" s="5"/>
     </row>
-    <row r="289" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="289" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A289" s="6"/>
       <c r="B289" s="6"/>
       <c r="C289" s="6"/>
@@ -9282,7 +9434,7 @@
       <c r="Y289" s="4"/>
       <c r="Z289" s="5"/>
     </row>
-    <row r="290" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="290" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A290" s="6"/>
       <c r="B290" s="6"/>
       <c r="C290" s="6"/>
@@ -9311,7 +9463,17 @@
       <c r="Z290" s="5"/>
     </row>
   </sheetData>
-  <mergeCells count="15">
+  <mergeCells count="18">
+    <mergeCell ref="A5:A10"/>
+    <mergeCell ref="C8:C10"/>
+    <mergeCell ref="D8:D10"/>
+    <mergeCell ref="B5:B7"/>
+    <mergeCell ref="C3:E3"/>
+    <mergeCell ref="E5:E7"/>
+    <mergeCell ref="B8:B10"/>
+    <mergeCell ref="E8:E10"/>
+    <mergeCell ref="C5:C7"/>
+    <mergeCell ref="D5:D7"/>
     <mergeCell ref="A1:Z1"/>
     <mergeCell ref="F2:J2"/>
     <mergeCell ref="K2:O2"/>
@@ -9320,14 +9482,13 @@
     <mergeCell ref="Q3:S3"/>
     <mergeCell ref="T3:V3"/>
     <mergeCell ref="W3:Y3"/>
-    <mergeCell ref="B5:B7"/>
-    <mergeCell ref="A5:A7"/>
-    <mergeCell ref="C3:E3"/>
-    <mergeCell ref="E5:E7"/>
-    <mergeCell ref="A8:A10"/>
-    <mergeCell ref="B8:B10"/>
-    <mergeCell ref="E8:E10"/>
   </mergeCells>
+  <phoneticPr fontId="12" type="noConversion"/>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B5:B10" xr:uid="{809D1943-C277-42AE-9640-1345005B66FC}">
+      <formula1>"Đào lò 1,Đào lò 2,Đào lò 3,Đào lò 6"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>

</xml_diff>